<commit_message>
Release v2.4.0 ODK XLSForm contract consolidation
</commit_message>
<xml_diff>
--- a/app/src/main/java/com/example/methodmesh/modules/appinspector/docs/example_odk_android_app_inspector.xlsx
+++ b/app/src/main/java/com/example/methodmesh/modules/appinspector/docs/example_odk_android_app_inspector.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rec19367c60684b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R7d8872a43f5447bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rac27b46266f841b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rc7012668674b474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R604cbb02f7b2487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rfa9c09b703144815"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +43,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -58,6 +58,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -93,7 +98,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -147,6 +152,25 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -584,28 +608,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="10" t="str">
+      <x:c r="A1" s="26" t="str">
         <x:v>form_title</x:v>
       </x:c>
-      <x:c r="B1" s="10" t="str">
+      <x:c r="B1" s="26" t="str">
         <x:v>form_id</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="26" t="str">
         <x:v>version</x:v>
       </x:c>
-      <x:c r="D1" s="10" t="str">
+      <x:c r="D1" s="26" t="str">
         <x:v>instance_name</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>android_app_inspector</x:v>
+        <x:v>Android App Inspector</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
         <x:v>android_app_inspector</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>2026072707</x:v>
+        <x:v>2026090703</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
         <x:v>${methodmesh_status}</x:v>

</xml_diff>